<commit_message>
Update handle database 2026-03-27
</commit_message>
<xml_diff>
--- a/carousel-data/handle-database.xlsx
+++ b/carousel-data/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4261,6 +4261,105 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>John Maxwell</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>The John Maxwell Company</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>johncmaxwell</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>@JohnCMaxwell</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>@johncmaxwell</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>@johncmaxwell</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>johnmaxwell</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Major leadership figure. X/Twitter and Instagram verified. No confirmed Bluesky or Threads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Dave Stachowiak</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Host, Coaching for Leaders podcast</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Coaching for Leaders</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>davestachowiak</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>@davestachowiak</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>X: VERIFIED, LinkedIn: VERIFIED. No IG/TikTok/YT/Threads/Bluesky found.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>